<commit_message>
Transcribe.ipynb - clean commit
</commit_message>
<xml_diff>
--- a/transcription_data/MCF_Languages.xlsx
+++ b/transcription_data/MCF_Languages.xlsx
@@ -1,78 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gayat\Desktop\transcription_script\transcription_data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB632260-71A0-4F72-BF69-24863D75DD23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Amharic" sheetId="1" r:id="rId1"/>
+    <sheet name="Amharic" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Audio_Samples</t>
-  </si>
-  <si>
-    <t>Original_transcript</t>
-  </si>
-  <si>
-    <t>Original_Translation</t>
-  </si>
-  <si>
-    <t>Match Percentage</t>
-  </si>
-  <si>
-    <t>Gemini _3.1_ Pro_Transcript</t>
-  </si>
-  <si>
-    <t>Gemini _3.1_ Pro_Translation</t>
-  </si>
-  <si>
-    <t>amharic_sample_1.wav</t>
-  </si>
-  <si>
-    <t>amharic_sample_2.wav</t>
-  </si>
-  <si>
-    <t>amharic_sample_3.wav</t>
-  </si>
-  <si>
-    <t>Аллаҳ, уи зыда Нцәа дыҟам иоуп. Иреиӷьӡоу ахьӡқәагьы Иара изкуп.</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -87,46 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -414,56 +420,170 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="20.33203125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="42.44140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="36.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="42" style="2" customWidth="1"/>
-    <col min="5" max="5" width="36.88671875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="18" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="2"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>3</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Audio_Samples</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Original_transcript</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Original_Translation</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Gemini _3.1_ Pro_Transcript</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Gemini _3.1_ Pro_Translation</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Match Percentage</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Gemini_3.1_Pro_Trancript</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Gemini_3.1_Pro_Translation</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Gemini_3.1_Pro_Match_Percentage</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Gemini_3.1_Pro_WER</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Gemini_3.1_Analysis</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
-      </c>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
-    <row r="4" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>7</v>
-      </c>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>amharic_sample_1.flac</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Аллаҳ, уи зыда Нцәа дыҟам иоуп. Иреиӷьӡоу ахьӡқәагьы Иара изкуп.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>በህዝብ ብዛት ከአፍሪካ ኢትዮጵያ ሁለተኛ ስትሆን በቆዳ ስፋት ደግሞ አስረኛ ናት።</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Ethiopia is second in Africa in population size, while it is tenth in land area.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
-    <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>8</v>
-      </c>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>amharic_sample_2.flac</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Арҭ шәара шәзы ҩныҵҟалагьы адәахьалагьы аҽрыцқьараз бжьгароуп.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>እነርሱም አዎ አሉት</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>And they said yes to him.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>amharic_sample_3.flac</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Абри, дара ирыҭоу, иҵабыргыҵәҟьоу ажәоуп.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>እንግዲያውማ ምስክር መሆን ካልቻልክ መጥተህ ክሳሳው እና እና ሙለታህን ከፍለንህ ሃብታም ትሆናለህ</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Well then, if you cannot be a witness, come and sue him, and we will repay your favor and you will become rich.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Percentage match with original script based on CER (Charater Error Recognition)
</commit_message>
<xml_diff>
--- a/transcription_data/MCF_Languages.xlsx
+++ b/transcription_data/MCF_Languages.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Amharic" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ligunda " sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +437,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Original_transcript</t>
+          <t>Original_Transcript</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -446,144 +447,316 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Gemini _3.1_ Pro_Transcript</t>
+          <t>Gemini_3.1_Pro_Trancript</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Gemini _3.1_ Pro_Translation</t>
+          <t>Gemini_3.1_Pro_Translation</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Match Percentage</t>
+          <t>Gemini_3.1_Pro_Match_Percentage</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Gemini_3.1_Pro_Trancript</t>
+          <t>Gemini_3.1_Pro_CER</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Gemini_3.1_Pro_Translation</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Gemini_3.1_Pro_Match_Percentage</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Gemini_3.1_Pro_WER</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Gemini_3.1_Analysis</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>amharic_sample_1.flac</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>"በህዝብ ብዛት ከአፍሪካ ኢትዮጵያ ሁለተኛ ስትሆን ፣ በቆዳ ስፋት ደግሞ አስረኛ ናት።"</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>"Ethiopia is the second most populous country in Africa, but the tenth largest in terms of land area."</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>በህዝብ ብዛት ከአፍሪካ ኢትዮጵያ ሁለተኛ ስትሆን በቆዳ ስፋት ደግሞ አስረኛ ናት።</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Ethiopia is second in Africa in population size, while it is tenth in land area.</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>The actual transcription quality is very high, featuring no missing words, no hallucinations, and perfectly retaining the correct meaning. The exceptionally low match score is misleading because the only difference is the omission of a single Amharic comma.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>amharic_sample_1.flac</t>
+          <t>amharic_sample_2.flac</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Аллаҳ, уи зыда Нцәа дыҟам иоуп. Иреиӷьӡоу ахьӡқәагьы Иара изкуп.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>በህዝብ ብዛት ከአፍሪካ ኢትዮጵያ ሁለተኛ ስትሆን በቆዳ ስፋት ደግሞ አስረኛ ናት።</t>
-        </is>
+          <t>"እነርሱም አዎ አሉት፡፡"</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>"And they said yes."</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>እነርሱም አዎ አሉት</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>And they said yes to him.</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>100</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Ethiopia is second in Africa in population size, while it is tenth in land area.</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+          <t>The transcription quality is practically perfect because it has no missing words, no incorrect meanings, and zero hallucinations. The artificially low match score is caused solely by the missing Amharic end punctuation (፡፡), even though the spoken words match exactly.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>amharic_sample_2.flac</t>
+          <t>amharic_sample_3.flac</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Арҭ шәара шәзы ҩныҵҟалагьы адәахьалагьы аҽрыцқьараз бжьгароуп.</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>እነርሱም አዎ አሉት</t>
-        </is>
+          <t>"እንግዲያውማ ምስክር መሆን ከቻልክ መጥተህ ክሰሰውና እናም ውለታህን ከፍለንህ ሃብታም ትሆናለህ፡፡"</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>"Then if you can be a witness, come and accuse him, and we will repay your favor and you will become rich."</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>እንግዲያውማ ምስክር መሆን ካልቻልክ መጥተህ ክሳሳው እና እና ሙለታህን ከፍለንህ ሃብታም ትሆናለህ</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Well then, if you cannot be a witness, come and sue him, and we will repay your favor and you will become rich.</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>85.70999999999999</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.1429</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>And they said yes to him.</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+          <t>The transcription quality is low primarily because changing "ከቻልክ" to "ካልቻልክ" completely reverses the sentence's meaning from "if you can" to "if you cannot". Instead of missing words, it hallucinates extra conjunctions and incorrectly transcribes "ክሰሰውና እናም ውለታህን" into the distorted phrase "ክሳሳው እና እና ሙለታህን".</t>
+        </is>
+      </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>amharic_sample_3.flac</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Абри, дара ирыҭоу, иҵабыргыҵәҟьоу ажәоуп.</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>እንግዲያውማ ምስክር መሆን ካልቻልክ መጥተህ ክሳሳው እና እና ሙለታህን ከፍለንህ ሃብታም ትሆናለህ</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Well then, if you cannot be a witness, come and sue him, and we will repay your favor and you will become rich.</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Audio_Samples</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Original_Transcript</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Original_Translation</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Gemini_3.1_Pro_Trancript</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Gemini_3.1_Pro_Translation</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Gemini_3.1_Pro_Match_Percentage</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Gemini_3.1_Pro_CER</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Gemini_3.1_Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ligunda_sample_1.wav</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Nze nnakoowa okukima amazzi kuba temunsasula buli lwe ngakima.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+I am tired of digging water because you don’t pay me every time I dig it.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nze nnakoowa okuwola kintu mmaawe nze kubanga temusasula buli lwe nkikima.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>I am tired of lending anything, my goodness, because you do not pay back every time I come to collect it.</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>66.04000000000001</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.3396</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>The transcription quality is extremely low because it hallucinates phrases like "okuwola kintu mmaawe" while missing key words like "okukima amazzi". These errors completely distort the sentence, resulting in an incorrect meaning that replaces the original context of fetching water with a nonsensical statement about lending things.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ligunda_sample_2.wav</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Neebaza nnyo ssezaala wange kuba yangabira ente.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+I am very grateful to my mother-in-law for giving me a cow.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Neebaza nnyo ssezaala wange kuba nga yampa ente</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>I thank my father-in-law very much because he gave me a cow.</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>85.37</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.1463</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Audio file 'ligunda_sample_2.wav' not found in Ligunda folder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ligunda_sample_3.wav</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ntudde nnyo kati omugongo gunnuma.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+I am sitting so much now my back hurts.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ntuudde nnyo kati omugongo gunnuma.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>I have been sitting for a long time, now my back hurts.</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>96.55</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0345</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Audio file 'ligunda_sample_3.wav' not found in Ligunda folder.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>